<commit_message>
Card - Deck update
</commit_message>
<xml_diff>
--- a/TSV Files/Warstcgv1.xlsx
+++ b/TSV Files/Warstcgv1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WARS TCG CARDS WORKING\WARS DRAGNCARDS PLUGIN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WARS TCG CARDS WORKING\WARS DRAGNCARDS PLUGIN\TSV Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58AA28DE-3DA5-4100-8C3D-82AFC0200DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A21785-73D5-4C39-B610-6104A8A366DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79FA9BEB-A46B-4836-B8C9-5D274259091F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79FA9BEB-A46B-4836-B8C9-5D274259091F}"/>
   </bookViews>
   <sheets>
     <sheet name="Warstcgv1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6282" uniqueCount="3102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7146" uniqueCount="3348">
   <si>
     <t>databaseId</t>
   </si>
@@ -9345,6 +9345,744 @@
   </si>
   <si>
     <t>normal</t>
+  </si>
+  <si>
+    <t>26aa24e6-4693-4aec-8b38-85f533f0b204</t>
+  </si>
+  <si>
+    <t>♦Horatio Hicks - WARS Tour</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F01.jpg</t>
+  </si>
+  <si>
+    <t>1F1</t>
+  </si>
+  <si>
+    <t>256a7a7b-bb54-459e-997d-16dbc940caf6</t>
+  </si>
+  <si>
+    <t>♦Jossel Swin</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01P01.jpg</t>
+  </si>
+  <si>
+    <t>1PF1</t>
+  </si>
+  <si>
+    <t>• Pay 3 energy ≈ This character is immune to attrition until end of turn. Each time you would reveal a card for battle destiny in a battle here, you may pay 3 energy. If you do, reveal three cards from the top of your reserve, choose one of them to add to your battle destiny instead, then put them on top of your used pile in any order.</t>
+  </si>
+  <si>
+    <t>A former squad leader, Swin was demoted when his hatred of the Mavericks manifested in extreme violence. Since the rift opened, his sanity has been in constant flux.</t>
+  </si>
+  <si>
+    <t>ff6852bd-ba2f-4d64-a75c-c838eea12f26</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R01.jpg</t>
+  </si>
+  <si>
+    <t>1RF1</t>
+  </si>
+  <si>
+    <t>f4cab8a3-41cd-470b-88ad-d0f81c6eacff</t>
+  </si>
+  <si>
+    <t>♦Kujiko Torako</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01P02.jpg</t>
+  </si>
+  <si>
+    <t>1PF2</t>
+  </si>
+  <si>
+    <t>CHARACTER • Kizen • Shikami • Unit</t>
+  </si>
+  <si>
+    <t>• Lose 2 energy ≈ This character is immune to attrition until end of turn. When this character enters play, you may play a unit here that costs 2 energy or less. That unit costs no energy to play.</t>
+  </si>
+  <si>
+    <t>“Understand. I still want to kill you. My duty requires I sublimate my desire.” - A Matter of Life or Death</t>
+  </si>
+  <si>
+    <t>1439b971-7952-4687-b741-56a20e9bb297</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R02.jpg</t>
+  </si>
+  <si>
+    <t>1RF2</t>
+  </si>
+  <si>
+    <t>31c69d01-b46a-42d0-9b12-f88221398d1b</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R03.jpg</t>
+  </si>
+  <si>
+    <t>1RF3</t>
+  </si>
+  <si>
+    <t>1161e6b2-f8ef-4bf0-b011-f38b458306a8</t>
+  </si>
+  <si>
+    <t>♦Talkan</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01P03.jpg</t>
+  </si>
+  <si>
+    <t>1PF3</t>
+  </si>
+  <si>
+    <t>• Put two cards from your hand on top of your used pile in any order ≈ This character is immune to attrition until end of turn. • Put target character you have here on top of its owner’s used pile ≈ Make this unit power +2 until end of turn.</t>
+  </si>
+  <si>
+    <t>Talkan assumed control of the Qurim tribe by killing the leader during ritual combat. His fury leads him into battle ahead of his troops.</t>
+  </si>
+  <si>
+    <t>88fb3fe5-7e7a-46de-8bd1-c03eb0298969</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R04.jpg</t>
+  </si>
+  <si>
+    <t>1RF4</t>
+  </si>
+  <si>
+    <t>4bbf5b5b-f03a-4206-9faa-e44c6bb39bd7</t>
+  </si>
+  <si>
+    <t>♦Ranarti-Anant</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01P04.jpg</t>
+  </si>
+  <si>
+    <t>1PF4</t>
+  </si>
+  <si>
+    <t>Piloting 3 (As long as this character is aboard a ship, that ship is power +3 and tactics +3.) • Dismiss target other unit you have here ≈ This character is immune to attrition until end of turn. • Pay 2 energy ≈ If this character is aboard a ship, move that ship to a sector battle at another sector.</t>
+  </si>
+  <si>
+    <t>A consummate pilot and wayfarer, Ranarti favors exploration over conflict. Its skills have brought it tremendous success in both endeavors.</t>
+  </si>
+  <si>
+    <t>91c0fa12-4278-4782-aa96-6435b72a57b7</t>
+  </si>
+  <si>
+    <t>State of Readiness - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F04.jpg</t>
+  </si>
+  <si>
+    <t>1F4</t>
+  </si>
+  <si>
+    <t>7b325dc4-5cce-4296-8555-63ce8301eeca</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R05.jpg</t>
+  </si>
+  <si>
+    <t>1RF5</t>
+  </si>
+  <si>
+    <t>80510dc5-044a-4ab3-91e7-cdb03f46ac72</t>
+  </si>
+  <si>
+    <t>Survey Cruiser - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F05.jpg</t>
+  </si>
+  <si>
+    <t>1F5</t>
+  </si>
+  <si>
+    <t>57d80fa8-df2d-4ffd-925e-f701c498bd39</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R06.jpg</t>
+  </si>
+  <si>
+    <t>1RF6</t>
+  </si>
+  <si>
+    <t>2337ae63-9573-43ad-a7cc-d7df345f2ea5</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R07.jpg</t>
+  </si>
+  <si>
+    <t>1RF7</t>
+  </si>
+  <si>
+    <t>3107540b-1b82-443f-8288-b1c768af5013</t>
+  </si>
+  <si>
+    <t>Cloud - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F07.jpg</t>
+  </si>
+  <si>
+    <t>1F7</t>
+  </si>
+  <si>
+    <t>a80edbdc-3c67-40c7-8af8-699e38b390af</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R08.jpg</t>
+  </si>
+  <si>
+    <t>1RF8</t>
+  </si>
+  <si>
+    <t>8b53dcc5-c87e-4ef7-8952-8de53fa82fbf</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R09.jpg</t>
+  </si>
+  <si>
+    <t>1RF9</t>
+  </si>
+  <si>
+    <t>2eceb65b-5385-416d-b6b8-19311179dd74</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R10.jpg</t>
+  </si>
+  <si>
+    <t>1RF10</t>
+  </si>
+  <si>
+    <t>0bd66106-5e1d-4501-9a2e-da03b1eb1cda</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R11.jpg</t>
+  </si>
+  <si>
+    <t>1RF11</t>
+  </si>
+  <si>
+    <t>0a209c37-ff30-4ecd-bcb9-f6dcee222abc</t>
+  </si>
+  <si>
+    <t>Loremaster - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F12.jpg</t>
+  </si>
+  <si>
+    <t>1F12</t>
+  </si>
+  <si>
+    <t>48f31ecd-94c3-495a-9ebb-626fd8d36379</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R12.jpg</t>
+  </si>
+  <si>
+    <t>1RF12</t>
+  </si>
+  <si>
+    <t>1d0eaf7c-819d-4451-8c50-498e36c81d35</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R13.jpg</t>
+  </si>
+  <si>
+    <t>1RF13</t>
+  </si>
+  <si>
+    <t>790864d4-dd31-46b0-a697-51c135bdcfda</t>
+  </si>
+  <si>
+    <t>♦Zocho - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F13.jpg</t>
+  </si>
+  <si>
+    <t>1F13</t>
+  </si>
+  <si>
+    <t>8a319d55-6155-4698-a4cf-b6ca80547b3e</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R14.jpg</t>
+  </si>
+  <si>
+    <t>1RF14</t>
+  </si>
+  <si>
+    <t>5aa3e397-5b18-486a-abdf-958b6f1a68c9</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R15.jpg</t>
+  </si>
+  <si>
+    <t>1RF15</t>
+  </si>
+  <si>
+    <t>2ffa8c85-4dbf-40a2-a4e8-bae085b27f4b</t>
+  </si>
+  <si>
+    <t>Fifth Ace - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F15.jpg</t>
+  </si>
+  <si>
+    <t>1F15</t>
+  </si>
+  <si>
+    <t>cecd85b0-acb2-4968-b311-148c25ed4f4f</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R16.jpg</t>
+  </si>
+  <si>
+    <t>1RF16</t>
+  </si>
+  <si>
+    <t>3be4f5f6-edc1-43be-b436-6e4b1fbb6fc3</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R17.jpg</t>
+  </si>
+  <si>
+    <t>1RF17</t>
+  </si>
+  <si>
+    <t>34817394-4d8d-43f6-aab5-ba2ea1a2fbec</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01R18.jpg</t>
+  </si>
+  <si>
+    <t>1RF18</t>
+  </si>
+  <si>
+    <t>2889b522-3c72-41e1-8185-b8f81ac580f5</t>
+  </si>
+  <si>
+    <t>Sultry Opportunist - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F18.jpg</t>
+  </si>
+  <si>
+    <t>1F18</t>
+  </si>
+  <si>
+    <t>b624ecb9-9083-4a0a-9c89-d71f2d70f443</t>
+  </si>
+  <si>
+    <t>♦Kulak - Essen Open Championship Oct 2004</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F19.jpg</t>
+  </si>
+  <si>
+    <t>1F19</t>
+  </si>
+  <si>
+    <t>a6eba5c4-7948-4b03-9089-c519e30c1dd1</t>
+  </si>
+  <si>
+    <t>Rally Cry - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F21.jpg</t>
+  </si>
+  <si>
+    <t>1F21</t>
+  </si>
+  <si>
+    <t>22b21a7b-2dd2-444d-a999-0adbd70dd02f</t>
+  </si>
+  <si>
+    <t>Revenge - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F22.jpg</t>
+  </si>
+  <si>
+    <t>1F22</t>
+  </si>
+  <si>
+    <t>20fbb651-5275-4353-9be3-62ba5a21c76c</t>
+  </si>
+  <si>
+    <t>Volt Scrounge - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F23.jpg</t>
+  </si>
+  <si>
+    <t>1F23</t>
+  </si>
+  <si>
+    <t>d60bcdbe-68b1-43d2-81cd-d73d468a8432</t>
+  </si>
+  <si>
+    <t>♦Devanar-Damir - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F24.jpg</t>
+  </si>
+  <si>
+    <t>1F24</t>
+  </si>
+  <si>
+    <t>1edc9d8d-a723-4f30-b064-b4e7497b1336</t>
+  </si>
+  <si>
+    <t>Selfless Protector - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F25.jpg</t>
+  </si>
+  <si>
+    <t>1F25</t>
+  </si>
+  <si>
+    <t>01dca171-3c0e-4c4c-bf83-ecb57db69d04</t>
+  </si>
+  <si>
+    <t>Expansion - WARS First Tournament Weekend Oct 2004</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F26.jpg</t>
+  </si>
+  <si>
+    <t>1F26</t>
+  </si>
+  <si>
+    <t>941e2593-e38d-4ab0-9646-395167482eea</t>
+  </si>
+  <si>
+    <t>Transport Depot - Rewards Store</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F27.jpg</t>
+  </si>
+  <si>
+    <t>1F27</t>
+  </si>
+  <si>
+    <t>5f19421a-55fa-46cd-aae1-c5976d6e9a9a</t>
+  </si>
+  <si>
+    <t>♦Ganymede/Traginium Well - Rewards Store</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F30.jpg</t>
+  </si>
+  <si>
+    <t>1F30</t>
+  </si>
+  <si>
+    <t>e3b05537-e1f3-47ea-9922-02882ded43a7</t>
+  </si>
+  <si>
+    <t>♦Ganymede/Underground Bunker - Rewards Store</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/1/WARS-EN01F31.jpg</t>
+  </si>
+  <si>
+    <t>1F31</t>
+  </si>
+  <si>
+    <t>610310b4-0838-4fd4-b5f1-c6e488868373</t>
+  </si>
+  <si>
+    <t>♦Dagger Lead</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02P01.jpg</t>
+  </si>
+  <si>
+    <t>2PF1</t>
+  </si>
+  <si>
+    <t>Size 2, Transport 1 • Invert this vehicle ≈ Undamage your target other unit in a site battle here./ Size 2, Transport 1</t>
+  </si>
+  <si>
+    <t>Howler’s command juggernaut has offspec mods the FedGrav designers never dreamed of.</t>
+  </si>
+  <si>
+    <t>47d2fa09-b48e-4ebf-b94a-46e7e9cabf19</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R01.jpg</t>
+  </si>
+  <si>
+    <t>2RF1</t>
+  </si>
+  <si>
+    <t>651afe2b-16c0-446a-993a-2467d3bb443c</t>
+  </si>
+  <si>
+    <t>Inca Fighter - Nowhere to Hide Pre-order incentive</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F01.jpg</t>
+  </si>
+  <si>
+    <t>2F1</t>
+  </si>
+  <si>
+    <t>efc0b32f-0a78-4899-8095-dbdd89d9c062</t>
+  </si>
+  <si>
+    <t>♦Killer Cait Grimalkin</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02P02.jpg</t>
+  </si>
+  <si>
+    <t>2PF2</t>
+  </si>
+  <si>
+    <t>Piloting 3 (As long as this character is aboard a ship, that ship is power +3 and tactics +3) • Pay 4 energy ≈ If this character is at a sector, your opponent can’t reveal cards for battle destiny during battles at target other sector until end of turn.</t>
+  </si>
+  <si>
+    <t>After all the cards are dealt, Killer Cait on your wing is better than pocket rockets.</t>
+  </si>
+  <si>
+    <t>1adf8480-a492-409f-8878-310cff7e6748</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R02.jpg</t>
+  </si>
+  <si>
+    <t>2RF2</t>
+  </si>
+  <si>
+    <t>b4fe0236-2ca1-4644-a1c2-b938896d9107</t>
+  </si>
+  <si>
+    <t>Ranger Watchman - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F02.jpg</t>
+  </si>
+  <si>
+    <t>2F2</t>
+  </si>
+  <si>
+    <t>910a42cc-4f81-4ef8-b633-b2c9d26a7daa</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R03.jpg</t>
+  </si>
+  <si>
+    <t>2RF3</t>
+  </si>
+  <si>
+    <t>c455de0b-16a6-4e01-bb28-9a6122fb5cf7</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R04.jpg</t>
+  </si>
+  <si>
+    <t>2RF4</t>
+  </si>
+  <si>
+    <t>c6c52703-6f3d-4639-aca3-17e5809a59d6</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R05.jpg</t>
+  </si>
+  <si>
+    <t>2RF5</t>
+  </si>
+  <si>
+    <t>e20fc04a-d8b9-4bc0-ac39-c075f5b0e4ee</t>
+  </si>
+  <si>
+    <t>Zhang Hotrod - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F05.jpg</t>
+  </si>
+  <si>
+    <t>2F5</t>
+  </si>
+  <si>
+    <t>09b5cfae-f206-4e7f-bc3a-110ceaa14ef2</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R06.jpg</t>
+  </si>
+  <si>
+    <t>2RF6</t>
+  </si>
+  <si>
+    <t>5a08155f-a188-40e0-afc6-944fe5783b19</t>
+  </si>
+  <si>
+    <t>Cornered - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F06.jpg</t>
+  </si>
+  <si>
+    <t>2F6</t>
+  </si>
+  <si>
+    <t>9be6fe1d-335c-46c0-b33e-28e86823638c</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R07.jpg</t>
+  </si>
+  <si>
+    <t>2RF7</t>
+  </si>
+  <si>
+    <t>NOBOT • Deigan • Inverter • Bot • Unit</t>
+  </si>
+  <si>
+    <t>9be49bbd-7382-4fc1-8f34-82bcca033d33</t>
+  </si>
+  <si>
+    <t>Lifeseeker - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F07.jpg</t>
+  </si>
+  <si>
+    <t>2F7</t>
+  </si>
+  <si>
+    <t>87317025-7eed-4a10-a099-51b56f06ffb0</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R08.jpg</t>
+  </si>
+  <si>
+    <t>2RF8</t>
+  </si>
+  <si>
+    <t>41a2be6e-0696-47ca-9d6c-07361ffc2cd0</t>
+  </si>
+  <si>
+    <t>♦Rakat - Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F09.jpg</t>
+  </si>
+  <si>
+    <t>2F9</t>
+  </si>
+  <si>
+    <t>7dd000fc-c8f2-4bf6-ab8c-67cc9716daa2</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R09.jpg</t>
+  </si>
+  <si>
+    <t>2RF9</t>
+  </si>
+  <si>
+    <t>129f53ee-1812-4501-a397-2646e701f14a</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R10.jpg</t>
+  </si>
+  <si>
+    <t>2RF10</t>
+  </si>
+  <si>
+    <t>c88418c7-8f18-4c42-a8f3-9272c8c579ae</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R11.jpg</t>
+  </si>
+  <si>
+    <t>2RF11</t>
+  </si>
+  <si>
+    <t>49a901e5-b32d-4397-9318-9e42b5f3adb4</t>
+  </si>
+  <si>
+    <t>Tahka Assault Craft- Starter Deck</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02F11.jpg</t>
+  </si>
+  <si>
+    <t>2F11</t>
+  </si>
+  <si>
+    <t>7aa0bbbb-0d00-4262-bb73-2ad0fdeb2548</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R12.jpg</t>
+  </si>
+  <si>
+    <t>2RF12</t>
+  </si>
+  <si>
+    <t>2bbbb46c-dae8-4dbd-b736-45475ba04592</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R13.jpg</t>
+  </si>
+  <si>
+    <t>2RF13</t>
+  </si>
+  <si>
+    <t>8bb041e6-a6c8-4aa3-8955-8cfa3fd9e56f</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R14.jpg</t>
+  </si>
+  <si>
+    <t>2RF14</t>
+  </si>
+  <si>
+    <t>0dbfd8fa-83a6-424d-8365-ea74fc060592</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R15.jpg</t>
+  </si>
+  <si>
+    <t>2RF15</t>
+  </si>
+  <si>
+    <t>a6bcb17f-538d-48d3-87e6-14b7b05ab934</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R16.jpg</t>
+  </si>
+  <si>
+    <t>2RF16</t>
+  </si>
+  <si>
+    <t>534c9a43-5c26-4b3a-9753-c76ea6533347</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R17.jpg</t>
+  </si>
+  <si>
+    <t>2RF17</t>
+  </si>
+  <si>
+    <t>6a1aa708-b234-441e-a285-f91fe7a30341</t>
+  </si>
+  <si>
+    <t>https://warstcg.org//img/2/WARS-EN02R18.jpg</t>
+  </si>
+  <si>
+    <t>2RF18</t>
   </si>
 </sst>
 </file>
@@ -9354,7 +10092,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9387,6 +10125,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -9405,10 +10151,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9425,8 +10172,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -9759,7 +10508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48FE8A57-0D3F-49E0-BA7C-D0804C020F31}">
-  <dimension ref="A1:T492"/>
+  <dimension ref="A1:T559"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.140625" customWidth="1"/>
@@ -37581,8 +38330,3875 @@
       </c>
       <c r="T492" s="7"/>
     </row>
+    <row r="493" spans="1:20" ht="15.75">
+      <c r="A493" s="9" t="s">
+        <v>3102</v>
+      </c>
+      <c r="B493" t="s">
+        <v>3103</v>
+      </c>
+      <c r="C493" s="10" t="s">
+        <v>3104</v>
+      </c>
+      <c r="D493" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E493" t="s">
+        <v>21</v>
+      </c>
+      <c r="F493" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G493" s="3">
+        <v>4</v>
+      </c>
+      <c r="H493" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I493" s="3" t="s">
+        <v>3105</v>
+      </c>
+      <c r="J493" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K493" t="s">
+        <v>85</v>
+      </c>
+      <c r="L493" s="3">
+        <v>5</v>
+      </c>
+      <c r="M493" s="3">
+        <v>3</v>
+      </c>
+      <c r="N493" t="s">
+        <v>28</v>
+      </c>
+      <c r="O493" s="3"/>
+      <c r="P493" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q493" s="3">
+        <v>6</v>
+      </c>
+      <c r="R493" s="3">
+        <v>4</v>
+      </c>
+      <c r="S493" t="s">
+        <v>86</v>
+      </c>
+      <c r="T493" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="494" spans="1:20" ht="15.75">
+      <c r="A494" t="s">
+        <v>3106</v>
+      </c>
+      <c r="B494" t="s">
+        <v>3107</v>
+      </c>
+      <c r="C494" t="s">
+        <v>3108</v>
+      </c>
+      <c r="D494" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E494" t="s">
+        <v>21</v>
+      </c>
+      <c r="F494" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G494" s="3">
+        <v>4</v>
+      </c>
+      <c r="H494" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I494" t="s">
+        <v>3109</v>
+      </c>
+      <c r="J494" t="s">
+        <v>8</v>
+      </c>
+      <c r="K494" t="s">
+        <v>773</v>
+      </c>
+      <c r="L494" s="3">
+        <v>2</v>
+      </c>
+      <c r="M494" s="3">
+        <v>5</v>
+      </c>
+      <c r="N494" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O494" s="3"/>
+      <c r="P494" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q494" s="3">
+        <v>3</v>
+      </c>
+      <c r="R494" s="3">
+        <v>5</v>
+      </c>
+      <c r="S494" t="s">
+        <v>3110</v>
+      </c>
+      <c r="T494" s="5" t="s">
+        <v>3111</v>
+      </c>
+    </row>
+    <row r="495" spans="1:20" ht="15.75">
+      <c r="A495" t="s">
+        <v>3112</v>
+      </c>
+      <c r="B495" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C495" t="s">
+        <v>3113</v>
+      </c>
+      <c r="D495" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E495" t="s">
+        <v>14</v>
+      </c>
+      <c r="F495" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G495" s="3">
+        <v>4</v>
+      </c>
+      <c r="H495" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I495" t="s">
+        <v>3114</v>
+      </c>
+      <c r="J495" t="s">
+        <v>8</v>
+      </c>
+      <c r="K495" t="s">
+        <v>18</v>
+      </c>
+      <c r="L495" s="3">
+        <v>2</v>
+      </c>
+      <c r="M495" s="3">
+        <v>3</v>
+      </c>
+      <c r="N495" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="O495" s="3"/>
+      <c r="P495" s="3"/>
+      <c r="Q495" s="3"/>
+      <c r="R495" s="3"/>
+      <c r="S495" t="s">
+        <v>40</v>
+      </c>
+      <c r="T495" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="496" spans="1:20" ht="15.75">
+      <c r="A496" t="s">
+        <v>3115</v>
+      </c>
+      <c r="B496" t="s">
+        <v>3116</v>
+      </c>
+      <c r="C496" t="s">
+        <v>3117</v>
+      </c>
+      <c r="D496" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E496" t="s">
+        <v>21</v>
+      </c>
+      <c r="F496" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G496" s="3">
+        <v>4</v>
+      </c>
+      <c r="H496" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I496" t="s">
+        <v>3118</v>
+      </c>
+      <c r="J496" t="s">
+        <v>149</v>
+      </c>
+      <c r="K496" t="s">
+        <v>3119</v>
+      </c>
+      <c r="L496" s="3">
+        <v>4</v>
+      </c>
+      <c r="M496" s="3">
+        <v>5</v>
+      </c>
+      <c r="N496" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="O496" s="3"/>
+      <c r="P496" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q496" s="3">
+        <v>4</v>
+      </c>
+      <c r="R496" s="3">
+        <v>6</v>
+      </c>
+      <c r="S496" t="s">
+        <v>3120</v>
+      </c>
+      <c r="T496" s="5" t="s">
+        <v>3121</v>
+      </c>
+    </row>
+    <row r="497" spans="1:20" ht="15.75">
+      <c r="A497" t="s">
+        <v>3122</v>
+      </c>
+      <c r="B497" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C497" t="s">
+        <v>3123</v>
+      </c>
+      <c r="D497" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E497" t="s">
+        <v>14</v>
+      </c>
+      <c r="F497" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G497" s="3">
+        <v>4</v>
+      </c>
+      <c r="H497" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I497" t="s">
+        <v>3124</v>
+      </c>
+      <c r="J497" t="s">
+        <v>8</v>
+      </c>
+      <c r="K497" t="s">
+        <v>18</v>
+      </c>
+      <c r="L497" s="3">
+        <v>3</v>
+      </c>
+      <c r="M497" s="3">
+        <v>5</v>
+      </c>
+      <c r="N497" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O497" s="3"/>
+      <c r="P497" s="3"/>
+      <c r="Q497" s="3"/>
+      <c r="R497" s="3"/>
+      <c r="S497" t="s">
+        <v>52</v>
+      </c>
+      <c r="T497" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="498" spans="1:20" ht="15.75">
+      <c r="A498" t="s">
+        <v>3125</v>
+      </c>
+      <c r="B498" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C498" t="s">
+        <v>3126</v>
+      </c>
+      <c r="D498" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E498" t="s">
+        <v>79</v>
+      </c>
+      <c r="F498" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G498" s="3">
+        <v>4</v>
+      </c>
+      <c r="H498" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I498" t="s">
+        <v>3127</v>
+      </c>
+      <c r="J498" t="s">
+        <v>8</v>
+      </c>
+      <c r="K498" t="s">
+        <v>80</v>
+      </c>
+      <c r="L498" s="3">
+        <v>4</v>
+      </c>
+      <c r="M498" s="3">
+        <v>2</v>
+      </c>
+      <c r="N498" t="s">
+        <v>11</v>
+      </c>
+      <c r="O498" s="3"/>
+      <c r="P498" s="3">
+        <v>8</v>
+      </c>
+      <c r="Q498" s="3">
+        <v>2</v>
+      </c>
+      <c r="R498" s="3">
+        <v>7</v>
+      </c>
+      <c r="S498" t="s">
+        <v>83</v>
+      </c>
+      <c r="T498" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="499" spans="1:20" ht="15.75">
+      <c r="A499" t="s">
+        <v>3128</v>
+      </c>
+      <c r="B499" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C499" t="s">
+        <v>3130</v>
+      </c>
+      <c r="D499" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E499" t="s">
+        <v>21</v>
+      </c>
+      <c r="F499" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G499" s="3">
+        <v>4</v>
+      </c>
+      <c r="H499" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I499" t="s">
+        <v>3131</v>
+      </c>
+      <c r="J499" t="s">
+        <v>557</v>
+      </c>
+      <c r="K499" t="s">
+        <v>1036</v>
+      </c>
+      <c r="L499" s="3">
+        <v>4</v>
+      </c>
+      <c r="M499" s="3">
+        <v>4</v>
+      </c>
+      <c r="N499" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="O499" s="3"/>
+      <c r="P499" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q499" s="3">
+        <v>2</v>
+      </c>
+      <c r="R499" s="3">
+        <v>6</v>
+      </c>
+      <c r="S499" t="s">
+        <v>3132</v>
+      </c>
+      <c r="T499" s="5" t="s">
+        <v>3133</v>
+      </c>
+    </row>
+    <row r="500" spans="1:20" ht="15.75">
+      <c r="A500" t="s">
+        <v>3134</v>
+      </c>
+      <c r="B500" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C500" t="s">
+        <v>3135</v>
+      </c>
+      <c r="D500" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E500" t="s">
+        <v>26</v>
+      </c>
+      <c r="F500" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G500" s="3">
+        <v>4</v>
+      </c>
+      <c r="H500" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I500" t="s">
+        <v>3136</v>
+      </c>
+      <c r="J500" t="s">
+        <v>8</v>
+      </c>
+      <c r="K500" t="s">
+        <v>47</v>
+      </c>
+      <c r="L500" s="3">
+        <v>2</v>
+      </c>
+      <c r="M500" s="3">
+        <v>4</v>
+      </c>
+      <c r="N500" t="s">
+        <v>23</v>
+      </c>
+      <c r="O500" s="3"/>
+      <c r="P500" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q500" s="3">
+        <v>1</v>
+      </c>
+      <c r="R500" s="3">
+        <v>5</v>
+      </c>
+      <c r="S500" t="s">
+        <v>91</v>
+      </c>
+      <c r="T500" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="501" spans="1:20" ht="15.75">
+      <c r="A501" t="s">
+        <v>3137</v>
+      </c>
+      <c r="B501" t="s">
+        <v>3138</v>
+      </c>
+      <c r="C501" t="s">
+        <v>3139</v>
+      </c>
+      <c r="D501" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E501" t="s">
+        <v>21</v>
+      </c>
+      <c r="F501" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G501" s="3">
+        <v>4</v>
+      </c>
+      <c r="H501" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I501" t="s">
+        <v>3140</v>
+      </c>
+      <c r="J501" t="s">
+        <v>426</v>
+      </c>
+      <c r="K501" t="s">
+        <v>972</v>
+      </c>
+      <c r="L501" s="3">
+        <v>4</v>
+      </c>
+      <c r="M501" s="3">
+        <v>5</v>
+      </c>
+      <c r="N501" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="O501" s="3"/>
+      <c r="P501" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q501" s="3">
+        <v>5</v>
+      </c>
+      <c r="R501" s="3">
+        <v>3</v>
+      </c>
+      <c r="S501" t="s">
+        <v>3141</v>
+      </c>
+      <c r="T501" s="5" t="s">
+        <v>3142</v>
+      </c>
+    </row>
+    <row r="502" spans="1:20" ht="15.75">
+      <c r="A502" t="s">
+        <v>3143</v>
+      </c>
+      <c r="B502" t="s">
+        <v>3144</v>
+      </c>
+      <c r="C502" t="s">
+        <v>3145</v>
+      </c>
+      <c r="D502" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E502" t="s">
+        <v>14</v>
+      </c>
+      <c r="F502" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G502" s="3">
+        <v>4</v>
+      </c>
+      <c r="H502" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I502" t="s">
+        <v>3146</v>
+      </c>
+      <c r="J502" t="s">
+        <v>8</v>
+      </c>
+      <c r="K502" t="s">
+        <v>15</v>
+      </c>
+      <c r="L502" s="3">
+        <v>1</v>
+      </c>
+      <c r="M502" s="3">
+        <v>2</v>
+      </c>
+      <c r="N502" t="s">
+        <v>23</v>
+      </c>
+      <c r="O502" s="3"/>
+      <c r="P502" s="3"/>
+      <c r="Q502" s="3"/>
+      <c r="R502" s="3"/>
+      <c r="S502" t="s">
+        <v>127</v>
+      </c>
+      <c r="T502" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="503" spans="1:20" ht="15.75">
+      <c r="A503" t="s">
+        <v>3147</v>
+      </c>
+      <c r="B503" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C503" t="s">
+        <v>3148</v>
+      </c>
+      <c r="D503" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E503" t="s">
+        <v>26</v>
+      </c>
+      <c r="F503" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G503" s="3">
+        <v>4</v>
+      </c>
+      <c r="H503" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I503" t="s">
+        <v>3149</v>
+      </c>
+      <c r="J503" t="s">
+        <v>8</v>
+      </c>
+      <c r="K503" t="s">
+        <v>47</v>
+      </c>
+      <c r="L503" s="3">
+        <v>3</v>
+      </c>
+      <c r="M503" s="3">
+        <v>6</v>
+      </c>
+      <c r="N503" t="s">
+        <v>11</v>
+      </c>
+      <c r="O503" s="3"/>
+      <c r="P503" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q503" s="3">
+        <v>1</v>
+      </c>
+      <c r="R503" s="3">
+        <v>5</v>
+      </c>
+      <c r="S503" t="s">
+        <v>93</v>
+      </c>
+      <c r="T503" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="504" spans="1:20" ht="15.75">
+      <c r="A504" t="s">
+        <v>3150</v>
+      </c>
+      <c r="B504" t="s">
+        <v>3151</v>
+      </c>
+      <c r="C504" t="s">
+        <v>3152</v>
+      </c>
+      <c r="D504" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E504" t="s">
+        <v>26</v>
+      </c>
+      <c r="F504" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G504" s="3">
+        <v>4</v>
+      </c>
+      <c r="H504" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I504" t="s">
+        <v>3153</v>
+      </c>
+      <c r="J504" t="s">
+        <v>8</v>
+      </c>
+      <c r="K504" t="s">
+        <v>60</v>
+      </c>
+      <c r="L504" s="3">
+        <v>5</v>
+      </c>
+      <c r="M504" s="3">
+        <v>1</v>
+      </c>
+      <c r="N504" t="s">
+        <v>11</v>
+      </c>
+      <c r="O504" s="3"/>
+      <c r="P504" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q504" s="3">
+        <v>2</v>
+      </c>
+      <c r="R504" s="3">
+        <v>8</v>
+      </c>
+      <c r="S504" t="s">
+        <v>131</v>
+      </c>
+      <c r="T504" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="505" spans="1:20" ht="15.75">
+      <c r="A505" t="s">
+        <v>3154</v>
+      </c>
+      <c r="B505" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C505" t="s">
+        <v>3155</v>
+      </c>
+      <c r="D505" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E505" t="s">
+        <v>21</v>
+      </c>
+      <c r="F505" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G505" s="3">
+        <v>4</v>
+      </c>
+      <c r="H505" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I505" t="s">
+        <v>3156</v>
+      </c>
+      <c r="J505" t="s">
+        <v>8</v>
+      </c>
+      <c r="K505" t="s">
+        <v>34</v>
+      </c>
+      <c r="L505" s="3">
+        <v>3</v>
+      </c>
+      <c r="M505" s="3">
+        <v>4</v>
+      </c>
+      <c r="N505" t="s">
+        <v>23</v>
+      </c>
+      <c r="O505" s="3"/>
+      <c r="P505" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q505" s="3">
+        <v>1</v>
+      </c>
+      <c r="R505" s="3">
+        <v>3</v>
+      </c>
+      <c r="S505" t="s">
+        <v>140</v>
+      </c>
+      <c r="T505" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="506" spans="1:20" ht="15.75">
+      <c r="A506" t="s">
+        <v>3157</v>
+      </c>
+      <c r="B506" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C506" t="s">
+        <v>3158</v>
+      </c>
+      <c r="D506" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E506" t="s">
+        <v>153</v>
+      </c>
+      <c r="F506" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G506" s="3">
+        <v>4</v>
+      </c>
+      <c r="H506" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I506" t="s">
+        <v>3159</v>
+      </c>
+      <c r="J506" t="s">
+        <v>149</v>
+      </c>
+      <c r="K506" t="s">
+        <v>154</v>
+      </c>
+      <c r="L506" s="3">
+        <v>0</v>
+      </c>
+      <c r="M506" s="3">
+        <v>4</v>
+      </c>
+      <c r="N506" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="O506" s="3"/>
+      <c r="P506" s="3"/>
+      <c r="Q506" s="3"/>
+      <c r="R506" s="3"/>
+      <c r="S506" t="s">
+        <v>155</v>
+      </c>
+      <c r="T506" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="507" spans="1:20" ht="15.75">
+      <c r="A507" t="s">
+        <v>3160</v>
+      </c>
+      <c r="B507" t="s">
+        <v>3161</v>
+      </c>
+      <c r="C507" t="s">
+        <v>3162</v>
+      </c>
+      <c r="D507" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E507" t="s">
+        <v>14</v>
+      </c>
+      <c r="F507" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G507" s="3">
+        <v>4</v>
+      </c>
+      <c r="H507" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I507" t="s">
+        <v>3163</v>
+      </c>
+      <c r="J507" t="s">
+        <v>149</v>
+      </c>
+      <c r="K507" t="s">
+        <v>18</v>
+      </c>
+      <c r="L507" s="3">
+        <v>0</v>
+      </c>
+      <c r="M507" s="3">
+        <v>6</v>
+      </c>
+      <c r="N507" t="s">
+        <v>167</v>
+      </c>
+      <c r="O507" s="3"/>
+      <c r="P507" s="3"/>
+      <c r="Q507" s="3"/>
+      <c r="R507" s="3"/>
+      <c r="S507" t="s">
+        <v>168</v>
+      </c>
+      <c r="T507" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="508" spans="1:20" ht="15.75">
+      <c r="A508" t="s">
+        <v>3164</v>
+      </c>
+      <c r="B508" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C508" t="s">
+        <v>3165</v>
+      </c>
+      <c r="D508" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E508" t="s">
+        <v>176</v>
+      </c>
+      <c r="F508" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G508" s="3">
+        <v>4</v>
+      </c>
+      <c r="H508" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I508" t="s">
+        <v>3166</v>
+      </c>
+      <c r="J508" t="s">
+        <v>149</v>
+      </c>
+      <c r="K508" t="s">
+        <v>177</v>
+      </c>
+      <c r="L508" s="3">
+        <v>6</v>
+      </c>
+      <c r="M508" s="3">
+        <v>5</v>
+      </c>
+      <c r="N508" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="O508" s="3"/>
+      <c r="P508" s="3">
+        <v>9</v>
+      </c>
+      <c r="Q508" s="3">
+        <v>4</v>
+      </c>
+      <c r="R508" s="3">
+        <v>5</v>
+      </c>
+      <c r="S508" t="s">
+        <v>178</v>
+      </c>
+      <c r="T508" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="509" spans="1:20" ht="15.75">
+      <c r="A509" t="s">
+        <v>3167</v>
+      </c>
+      <c r="B509" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C509" t="s">
+        <v>3168</v>
+      </c>
+      <c r="D509" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E509" t="s">
+        <v>176</v>
+      </c>
+      <c r="F509" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G509" s="3">
+        <v>4</v>
+      </c>
+      <c r="H509" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I509" t="s">
+        <v>3169</v>
+      </c>
+      <c r="J509" t="s">
+        <v>149</v>
+      </c>
+      <c r="K509" t="s">
+        <v>205</v>
+      </c>
+      <c r="L509" s="3">
+        <v>5</v>
+      </c>
+      <c r="M509" s="3">
+        <v>3</v>
+      </c>
+      <c r="N509" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="O509" s="3"/>
+      <c r="P509" s="3">
+        <v>8</v>
+      </c>
+      <c r="Q509" s="3">
+        <v>2</v>
+      </c>
+      <c r="R509" s="3">
+        <v>8</v>
+      </c>
+      <c r="S509" t="s">
+        <v>206</v>
+      </c>
+      <c r="T509" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="510" spans="1:20" ht="15.75">
+      <c r="A510" t="s">
+        <v>3170</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1215</v>
+      </c>
+      <c r="C510" t="s">
+        <v>3171</v>
+      </c>
+      <c r="D510" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E510" t="s">
+        <v>9</v>
+      </c>
+      <c r="F510" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G510" s="3">
+        <v>4</v>
+      </c>
+      <c r="H510" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I510" t="s">
+        <v>3172</v>
+      </c>
+      <c r="J510" t="s">
+        <v>149</v>
+      </c>
+      <c r="K510" t="s">
+        <v>116</v>
+      </c>
+      <c r="L510" s="3">
+        <v>2</v>
+      </c>
+      <c r="M510" s="3">
+        <v>0</v>
+      </c>
+      <c r="N510" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="O510" s="3"/>
+      <c r="P510" s="3"/>
+      <c r="Q510" s="3"/>
+      <c r="R510" s="3"/>
+      <c r="S510" t="s">
+        <v>231</v>
+      </c>
+      <c r="T510" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="511" spans="1:20" ht="15.75">
+      <c r="A511" t="s">
+        <v>3173</v>
+      </c>
+      <c r="B511" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C511" t="s">
+        <v>3174</v>
+      </c>
+      <c r="D511" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E511" t="s">
+        <v>176</v>
+      </c>
+      <c r="F511" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G511" s="3">
+        <v>4</v>
+      </c>
+      <c r="H511" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I511" t="s">
+        <v>3175</v>
+      </c>
+      <c r="J511" t="s">
+        <v>149</v>
+      </c>
+      <c r="K511" t="s">
+        <v>257</v>
+      </c>
+      <c r="L511" s="3">
+        <v>6</v>
+      </c>
+      <c r="M511" s="3">
+        <v>3</v>
+      </c>
+      <c r="N511" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="O511" s="3"/>
+      <c r="P511" s="3">
+        <v>7</v>
+      </c>
+      <c r="Q511" s="3">
+        <v>3</v>
+      </c>
+      <c r="R511" s="3">
+        <v>6</v>
+      </c>
+      <c r="S511" t="s">
+        <v>258</v>
+      </c>
+      <c r="T511" s="5" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="512" spans="1:20" ht="15.75">
+      <c r="A512" t="s">
+        <v>3176</v>
+      </c>
+      <c r="B512" t="s">
+        <v>3177</v>
+      </c>
+      <c r="C512" t="s">
+        <v>3178</v>
+      </c>
+      <c r="D512" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E512" t="s">
+        <v>21</v>
+      </c>
+      <c r="F512" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G512" s="3">
+        <v>4</v>
+      </c>
+      <c r="H512" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I512" t="s">
+        <v>3179</v>
+      </c>
+      <c r="J512" t="s">
+        <v>149</v>
+      </c>
+      <c r="K512" t="s">
+        <v>164</v>
+      </c>
+      <c r="L512" s="3">
+        <v>2</v>
+      </c>
+      <c r="M512" s="3">
+        <v>4</v>
+      </c>
+      <c r="N512" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="O512" s="3"/>
+      <c r="P512" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q512" s="3">
+        <v>2</v>
+      </c>
+      <c r="R512" s="3">
+        <v>1</v>
+      </c>
+      <c r="S512" t="s">
+        <v>229</v>
+      </c>
+      <c r="T512" s="5" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="513" spans="1:20" ht="15.75">
+      <c r="A513" t="s">
+        <v>3180</v>
+      </c>
+      <c r="B513" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C513" t="s">
+        <v>3181</v>
+      </c>
+      <c r="D513" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E513" t="s">
+        <v>153</v>
+      </c>
+      <c r="F513" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G513" s="3">
+        <v>4</v>
+      </c>
+      <c r="H513" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I513" t="s">
+        <v>3182</v>
+      </c>
+      <c r="J513" t="s">
+        <v>287</v>
+      </c>
+      <c r="K513" t="s">
+        <v>353</v>
+      </c>
+      <c r="L513" s="3">
+        <v>1</v>
+      </c>
+      <c r="M513" s="3">
+        <v>5</v>
+      </c>
+      <c r="N513" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="O513" s="3"/>
+      <c r="P513" s="3"/>
+      <c r="Q513" s="3"/>
+      <c r="R513" s="3"/>
+      <c r="S513" t="s">
+        <v>354</v>
+      </c>
+      <c r="T513" s="5" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="514" spans="1:20" ht="15.75">
+      <c r="A514" t="s">
+        <v>3183</v>
+      </c>
+      <c r="B514" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C514" t="s">
+        <v>3184</v>
+      </c>
+      <c r="D514" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E514" t="s">
+        <v>21</v>
+      </c>
+      <c r="F514" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G514" s="3">
+        <v>4</v>
+      </c>
+      <c r="H514" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I514" t="s">
+        <v>3185</v>
+      </c>
+      <c r="J514" t="s">
+        <v>287</v>
+      </c>
+      <c r="K514" t="s">
+        <v>407</v>
+      </c>
+      <c r="L514" s="3">
+        <v>3</v>
+      </c>
+      <c r="M514" s="3">
+        <v>5</v>
+      </c>
+      <c r="N514" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="O514" s="3"/>
+      <c r="P514" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q514" s="3">
+        <v>5</v>
+      </c>
+      <c r="R514" s="3">
+        <v>6</v>
+      </c>
+      <c r="S514" t="s">
+        <v>408</v>
+      </c>
+      <c r="T514" s="5" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="515" spans="1:20" ht="15.75">
+      <c r="A515" t="s">
+        <v>3186</v>
+      </c>
+      <c r="B515" t="s">
+        <v>3187</v>
+      </c>
+      <c r="C515" t="s">
+        <v>3188</v>
+      </c>
+      <c r="D515" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E515" t="s">
+        <v>26</v>
+      </c>
+      <c r="F515" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G515" s="3">
+        <v>4</v>
+      </c>
+      <c r="H515" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I515" t="s">
+        <v>3189</v>
+      </c>
+      <c r="J515" t="s">
+        <v>149</v>
+      </c>
+      <c r="K515" t="s">
+        <v>194</v>
+      </c>
+      <c r="L515" s="3">
+        <v>4</v>
+      </c>
+      <c r="M515" s="3">
+        <v>1</v>
+      </c>
+      <c r="N515" t="s">
+        <v>167</v>
+      </c>
+      <c r="O515" s="3"/>
+      <c r="P515" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q515" s="3">
+        <v>3</v>
+      </c>
+      <c r="R515" s="3">
+        <v>5</v>
+      </c>
+      <c r="S515" t="s">
+        <v>283</v>
+      </c>
+      <c r="T515" s="5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="516" spans="1:20" ht="15.75">
+      <c r="A516" t="s">
+        <v>3190</v>
+      </c>
+      <c r="B516" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C516" t="s">
+        <v>3191</v>
+      </c>
+      <c r="D516" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E516" t="s">
+        <v>21</v>
+      </c>
+      <c r="F516" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G516" s="3">
+        <v>4</v>
+      </c>
+      <c r="H516" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I516" t="s">
+        <v>3192</v>
+      </c>
+      <c r="J516" t="s">
+        <v>287</v>
+      </c>
+      <c r="K516" t="s">
+        <v>420</v>
+      </c>
+      <c r="L516" s="3">
+        <v>2</v>
+      </c>
+      <c r="M516" s="3">
+        <v>2</v>
+      </c>
+      <c r="N516" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="O516" s="3"/>
+      <c r="P516" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q516" s="3">
+        <v>3</v>
+      </c>
+      <c r="R516" s="3">
+        <v>2</v>
+      </c>
+      <c r="S516" t="s">
+        <v>421</v>
+      </c>
+      <c r="T516" s="5" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="517" spans="1:20" ht="15.75">
+      <c r="A517" t="s">
+        <v>3193</v>
+      </c>
+      <c r="B517" t="s">
+        <v>1350</v>
+      </c>
+      <c r="C517" t="s">
+        <v>3194</v>
+      </c>
+      <c r="D517" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E517" t="s">
+        <v>21</v>
+      </c>
+      <c r="F517" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G517" s="3">
+        <v>4</v>
+      </c>
+      <c r="H517" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I517" t="s">
+        <v>3195</v>
+      </c>
+      <c r="J517" t="s">
+        <v>557</v>
+      </c>
+      <c r="K517" t="s">
+        <v>561</v>
+      </c>
+      <c r="L517" s="3">
+        <v>2</v>
+      </c>
+      <c r="M517" s="3">
+        <v>2</v>
+      </c>
+      <c r="N517" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="O517" s="3"/>
+      <c r="P517" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q517" s="3">
+        <v>1</v>
+      </c>
+      <c r="R517" s="3">
+        <v>3</v>
+      </c>
+      <c r="S517" t="s">
+        <v>562</v>
+      </c>
+      <c r="T517" s="5" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="518" spans="1:20" ht="15.75">
+      <c r="A518" t="s">
+        <v>3196</v>
+      </c>
+      <c r="B518" t="s">
+        <v>3197</v>
+      </c>
+      <c r="C518" t="s">
+        <v>3198</v>
+      </c>
+      <c r="D518" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E518" t="s">
+        <v>14</v>
+      </c>
+      <c r="F518" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G518" s="3">
+        <v>4</v>
+      </c>
+      <c r="H518" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I518" t="s">
+        <v>3199</v>
+      </c>
+      <c r="J518" t="s">
+        <v>287</v>
+      </c>
+      <c r="K518" t="s">
+        <v>15</v>
+      </c>
+      <c r="L518" s="3">
+        <v>3</v>
+      </c>
+      <c r="M518" s="3">
+        <v>5</v>
+      </c>
+      <c r="N518" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="O518" s="3"/>
+      <c r="P518" s="3"/>
+      <c r="Q518" s="3"/>
+      <c r="R518" s="3"/>
+      <c r="S518" t="s">
+        <v>325</v>
+      </c>
+      <c r="T518" s="5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="519" spans="1:20" ht="15.75">
+      <c r="A519" t="s">
+        <v>3200</v>
+      </c>
+      <c r="B519" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C519" t="s">
+        <v>3201</v>
+      </c>
+      <c r="D519" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E519" t="s">
+        <v>9</v>
+      </c>
+      <c r="F519" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G519" s="3">
+        <v>4</v>
+      </c>
+      <c r="H519" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I519" t="s">
+        <v>3202</v>
+      </c>
+      <c r="J519" t="s">
+        <v>557</v>
+      </c>
+      <c r="K519" t="s">
+        <v>9</v>
+      </c>
+      <c r="L519" s="3">
+        <v>3</v>
+      </c>
+      <c r="M519" s="3">
+        <v>3</v>
+      </c>
+      <c r="N519" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="O519" s="3"/>
+      <c r="P519" s="3"/>
+      <c r="Q519" s="3"/>
+      <c r="R519" s="3"/>
+      <c r="S519" t="s">
+        <v>574</v>
+      </c>
+      <c r="T519" s="5" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="520" spans="1:20" ht="15.75">
+      <c r="A520" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B520" t="s">
+        <v>1394</v>
+      </c>
+      <c r="C520" t="s">
+        <v>3204</v>
+      </c>
+      <c r="D520" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E520" t="s">
+        <v>14</v>
+      </c>
+      <c r="F520" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G520" s="3">
+        <v>4</v>
+      </c>
+      <c r="H520" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I520" t="s">
+        <v>3205</v>
+      </c>
+      <c r="J520" t="s">
+        <v>557</v>
+      </c>
+      <c r="K520" t="s">
+        <v>18</v>
+      </c>
+      <c r="L520" s="3">
+        <v>3</v>
+      </c>
+      <c r="M520" s="3">
+        <v>2</v>
+      </c>
+      <c r="N520" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="O520" s="3"/>
+      <c r="P520" s="3"/>
+      <c r="Q520" s="3"/>
+      <c r="R520" s="3"/>
+      <c r="S520" t="s">
+        <v>672</v>
+      </c>
+      <c r="T520" s="5" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="521" spans="1:20" ht="15.75">
+      <c r="A521" t="s">
+        <v>3206</v>
+      </c>
+      <c r="B521" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C521" t="s">
+        <v>3207</v>
+      </c>
+      <c r="D521" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E521" t="s">
+        <v>14</v>
+      </c>
+      <c r="F521" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G521" s="3">
+        <v>4</v>
+      </c>
+      <c r="H521" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I521" t="s">
+        <v>3208</v>
+      </c>
+      <c r="J521" t="s">
+        <v>426</v>
+      </c>
+      <c r="K521" t="s">
+        <v>18</v>
+      </c>
+      <c r="L521" s="3">
+        <v>0</v>
+      </c>
+      <c r="M521" s="3">
+        <v>6</v>
+      </c>
+      <c r="N521" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="O521" s="3"/>
+      <c r="P521" s="3"/>
+      <c r="Q521" s="3"/>
+      <c r="R521" s="3"/>
+      <c r="S521" t="s">
+        <v>465</v>
+      </c>
+      <c r="T521" s="5" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="522" spans="1:20" ht="15.75">
+      <c r="A522" t="s">
+        <v>3209</v>
+      </c>
+      <c r="B522" t="s">
+        <v>3210</v>
+      </c>
+      <c r="C522" t="s">
+        <v>3211</v>
+      </c>
+      <c r="D522" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E522" t="s">
+        <v>21</v>
+      </c>
+      <c r="F522" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G522" s="3">
+        <v>4</v>
+      </c>
+      <c r="H522" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I522" t="s">
+        <v>3212</v>
+      </c>
+      <c r="J522" t="s">
+        <v>287</v>
+      </c>
+      <c r="K522" t="s">
+        <v>316</v>
+      </c>
+      <c r="L522" s="3">
+        <v>1</v>
+      </c>
+      <c r="M522" s="3">
+        <v>3</v>
+      </c>
+      <c r="N522" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="O522" s="3"/>
+      <c r="P522" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q522" s="3">
+        <v>1</v>
+      </c>
+      <c r="R522" s="3">
+        <v>4</v>
+      </c>
+      <c r="S522" t="s">
+        <v>405</v>
+      </c>
+      <c r="T522" s="5" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="523" spans="1:20" ht="15.75">
+      <c r="A523" t="s">
+        <v>3213</v>
+      </c>
+      <c r="B523" t="s">
+        <v>3214</v>
+      </c>
+      <c r="C523" t="s">
+        <v>3215</v>
+      </c>
+      <c r="D523" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E523" t="s">
+        <v>21</v>
+      </c>
+      <c r="F523" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G523" s="3">
+        <v>4</v>
+      </c>
+      <c r="H523" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I523" t="s">
+        <v>3216</v>
+      </c>
+      <c r="J523" t="s">
+        <v>557</v>
+      </c>
+      <c r="K523" t="s">
+        <v>616</v>
+      </c>
+      <c r="L523" s="3">
+        <v>4</v>
+      </c>
+      <c r="M523" s="3">
+        <v>4</v>
+      </c>
+      <c r="N523" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="O523" s="3"/>
+      <c r="P523" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q523" s="3">
+        <v>4</v>
+      </c>
+      <c r="R523" s="3">
+        <v>6</v>
+      </c>
+      <c r="S523" t="s">
+        <v>617</v>
+      </c>
+      <c r="T523" s="5" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="524" spans="1:20" ht="15.75">
+      <c r="A524" t="s">
+        <v>3217</v>
+      </c>
+      <c r="B524" t="s">
+        <v>3218</v>
+      </c>
+      <c r="C524" t="s">
+        <v>3219</v>
+      </c>
+      <c r="D524" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E524" t="s">
+        <v>9</v>
+      </c>
+      <c r="F524" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G524" s="3">
+        <v>4</v>
+      </c>
+      <c r="H524" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I524" t="s">
+        <v>3220</v>
+      </c>
+      <c r="J524" t="s">
+        <v>557</v>
+      </c>
+      <c r="K524" t="s">
+        <v>9</v>
+      </c>
+      <c r="L524" s="3">
+        <v>1</v>
+      </c>
+      <c r="M524" s="3">
+        <v>2</v>
+      </c>
+      <c r="N524" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="O524" s="3"/>
+      <c r="P524" s="3"/>
+      <c r="Q524" s="3"/>
+      <c r="R524" s="3"/>
+      <c r="S524" t="s">
+        <v>653</v>
+      </c>
+      <c r="T524" s="5" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="525" spans="1:20" ht="15.75">
+      <c r="A525" t="s">
+        <v>3221</v>
+      </c>
+      <c r="B525" t="s">
+        <v>3222</v>
+      </c>
+      <c r="C525" t="s">
+        <v>3223</v>
+      </c>
+      <c r="D525" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E525" t="s">
+        <v>14</v>
+      </c>
+      <c r="F525" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G525" s="3">
+        <v>4</v>
+      </c>
+      <c r="H525" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I525" t="s">
+        <v>3224</v>
+      </c>
+      <c r="J525" t="s">
+        <v>557</v>
+      </c>
+      <c r="K525" t="s">
+        <v>18</v>
+      </c>
+      <c r="L525" s="3">
+        <v>2</v>
+      </c>
+      <c r="M525" s="3">
+        <v>4</v>
+      </c>
+      <c r="N525" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="O525" s="3"/>
+      <c r="P525" s="3"/>
+      <c r="Q525" s="3"/>
+      <c r="R525" s="3"/>
+      <c r="S525" t="s">
+        <v>660</v>
+      </c>
+      <c r="T525" s="5" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="526" spans="1:20" ht="15.75">
+      <c r="A526" t="s">
+        <v>3225</v>
+      </c>
+      <c r="B526" t="s">
+        <v>3226</v>
+      </c>
+      <c r="C526" t="s">
+        <v>3227</v>
+      </c>
+      <c r="D526" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E526" t="s">
+        <v>21</v>
+      </c>
+      <c r="F526" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G526" s="3">
+        <v>4</v>
+      </c>
+      <c r="H526" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I526" t="s">
+        <v>3228</v>
+      </c>
+      <c r="J526" t="s">
+        <v>557</v>
+      </c>
+      <c r="K526" t="s">
+        <v>566</v>
+      </c>
+      <c r="L526" s="3">
+        <v>4</v>
+      </c>
+      <c r="M526" s="3">
+        <v>2</v>
+      </c>
+      <c r="N526" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="O526" s="3"/>
+      <c r="P526" s="6">
+        <v>43862</v>
+      </c>
+      <c r="Q526" s="6">
+        <v>43925</v>
+      </c>
+      <c r="R526" s="6">
+        <v>43983</v>
+      </c>
+      <c r="S526" t="s">
+        <v>689</v>
+      </c>
+      <c r="T526" s="5" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="527" spans="1:20" ht="15.75">
+      <c r="A527" t="s">
+        <v>3229</v>
+      </c>
+      <c r="B527" t="s">
+        <v>3230</v>
+      </c>
+      <c r="C527" t="s">
+        <v>3231</v>
+      </c>
+      <c r="D527" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E527" t="s">
+        <v>21</v>
+      </c>
+      <c r="F527" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G527" s="3">
+        <v>4</v>
+      </c>
+      <c r="H527" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I527" t="s">
+        <v>3232</v>
+      </c>
+      <c r="J527" t="s">
+        <v>426</v>
+      </c>
+      <c r="K527" t="s">
+        <v>451</v>
+      </c>
+      <c r="L527" s="3">
+        <v>4</v>
+      </c>
+      <c r="M527" s="3">
+        <v>1</v>
+      </c>
+      <c r="N527" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="O527" s="3"/>
+      <c r="P527" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q527" s="3">
+        <v>3</v>
+      </c>
+      <c r="R527" s="3">
+        <v>5</v>
+      </c>
+      <c r="S527" t="s">
+        <v>459</v>
+      </c>
+      <c r="T527" s="5" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="528" spans="1:20" ht="15.75">
+      <c r="A528" t="s">
+        <v>3233</v>
+      </c>
+      <c r="B528" t="s">
+        <v>3234</v>
+      </c>
+      <c r="C528" t="s">
+        <v>3235</v>
+      </c>
+      <c r="D528" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E528" t="s">
+        <v>21</v>
+      </c>
+      <c r="F528" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G528" s="3">
+        <v>60</v>
+      </c>
+      <c r="H528" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I528" t="s">
+        <v>3236</v>
+      </c>
+      <c r="J528" t="s">
+        <v>426</v>
+      </c>
+      <c r="K528" t="s">
+        <v>515</v>
+      </c>
+      <c r="L528" s="3">
+        <v>1</v>
+      </c>
+      <c r="M528" s="3">
+        <v>5</v>
+      </c>
+      <c r="N528" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="O528" s="3"/>
+      <c r="P528" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q528" s="3">
+        <v>2</v>
+      </c>
+      <c r="R528" s="3">
+        <v>5</v>
+      </c>
+      <c r="S528" t="s">
+        <v>516</v>
+      </c>
+      <c r="T528" s="5" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="529" spans="1:20" ht="15.75">
+      <c r="A529" t="s">
+        <v>3237</v>
+      </c>
+      <c r="B529" t="s">
+        <v>3238</v>
+      </c>
+      <c r="C529" t="s">
+        <v>3239</v>
+      </c>
+      <c r="D529" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E529" t="s">
+        <v>14</v>
+      </c>
+      <c r="F529" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G529" s="3">
+        <v>60</v>
+      </c>
+      <c r="H529" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I529" t="s">
+        <v>3240</v>
+      </c>
+      <c r="J529" t="s">
+        <v>693</v>
+      </c>
+      <c r="K529" t="s">
+        <v>18</v>
+      </c>
+      <c r="L529" s="3">
+        <v>0</v>
+      </c>
+      <c r="M529" s="3">
+        <v>3</v>
+      </c>
+      <c r="N529" s="4"/>
+      <c r="O529" s="3"/>
+      <c r="P529" s="3"/>
+      <c r="Q529" s="3"/>
+      <c r="R529" s="3"/>
+      <c r="S529" t="s">
+        <v>706</v>
+      </c>
+      <c r="T529" s="5" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="530" spans="1:20" ht="15.75">
+      <c r="A530" s="9" t="s">
+        <v>3241</v>
+      </c>
+      <c r="B530" t="s">
+        <v>3242</v>
+      </c>
+      <c r="C530" t="s">
+        <v>3243</v>
+      </c>
+      <c r="D530" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E530" t="s">
+        <v>9</v>
+      </c>
+      <c r="F530" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G530" s="3">
+        <v>60</v>
+      </c>
+      <c r="H530" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I530" t="s">
+        <v>3244</v>
+      </c>
+      <c r="J530" t="s">
+        <v>693</v>
+      </c>
+      <c r="K530" t="s">
+        <v>31</v>
+      </c>
+      <c r="L530" s="3">
+        <v>1</v>
+      </c>
+      <c r="M530" s="3">
+        <v>5</v>
+      </c>
+      <c r="N530" s="4"/>
+      <c r="O530" s="3"/>
+      <c r="P530" s="3"/>
+      <c r="Q530" s="3"/>
+      <c r="R530" s="3"/>
+      <c r="S530" t="s">
+        <v>729</v>
+      </c>
+      <c r="T530" s="5" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="531" spans="1:20" ht="15.75">
+      <c r="A531" t="s">
+        <v>3245</v>
+      </c>
+      <c r="B531" t="s">
+        <v>3246</v>
+      </c>
+      <c r="C531" t="s">
+        <v>3247</v>
+      </c>
+      <c r="D531" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E531" t="s">
+        <v>3098</v>
+      </c>
+      <c r="F531" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G531" s="3">
+        <v>4</v>
+      </c>
+      <c r="H531" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I531" t="s">
+        <v>3248</v>
+      </c>
+      <c r="K531" t="s">
+        <v>736</v>
+      </c>
+      <c r="L531" s="3">
+        <v>0</v>
+      </c>
+      <c r="M531" s="3">
+        <v>3</v>
+      </c>
+      <c r="N531" s="4"/>
+      <c r="O531" s="6">
+        <v>43863</v>
+      </c>
+      <c r="P531" s="3"/>
+      <c r="Q531" s="3"/>
+      <c r="R531" s="3"/>
+      <c r="S531" t="s">
+        <v>754</v>
+      </c>
+      <c r="T531" s="7"/>
+    </row>
+    <row r="532" spans="1:20" ht="15.75">
+      <c r="A532" t="s">
+        <v>3249</v>
+      </c>
+      <c r="B532" t="s">
+        <v>3250</v>
+      </c>
+      <c r="C532" t="s">
+        <v>3251</v>
+      </c>
+      <c r="D532" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E532" t="s">
+        <v>3098</v>
+      </c>
+      <c r="F532" s="3" t="s">
+        <v>2112</v>
+      </c>
+      <c r="G532" s="3">
+        <v>4</v>
+      </c>
+      <c r="H532" t="s">
+        <v>3096</v>
+      </c>
+      <c r="I532" t="s">
+        <v>3252</v>
+      </c>
+      <c r="K532" t="s">
+        <v>751</v>
+      </c>
+      <c r="L532" s="3">
+        <v>0</v>
+      </c>
+      <c r="M532" s="3">
+        <v>0</v>
+      </c>
+      <c r="N532" t="s">
+        <v>167</v>
+      </c>
+      <c r="O532" s="6">
+        <v>43862</v>
+      </c>
+      <c r="P532" s="3"/>
+      <c r="Q532" s="3"/>
+      <c r="R532" s="3"/>
+      <c r="S532" t="s">
+        <v>755</v>
+      </c>
+      <c r="T532" s="7"/>
+    </row>
+    <row r="533" spans="1:20" ht="15.75">
+      <c r="A533" t="s">
+        <v>3253</v>
+      </c>
+      <c r="B533" t="s">
+        <v>3254</v>
+      </c>
+      <c r="C533" t="s">
+        <v>3255</v>
+      </c>
+      <c r="D533" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E533" t="s">
+        <v>79</v>
+      </c>
+      <c r="F533" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G533" s="3">
+        <v>4</v>
+      </c>
+      <c r="H533" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I533" t="s">
+        <v>3256</v>
+      </c>
+      <c r="J533" t="s">
+        <v>8</v>
+      </c>
+      <c r="K533" t="s">
+        <v>778</v>
+      </c>
+      <c r="L533" s="3">
+        <v>6</v>
+      </c>
+      <c r="M533" s="3">
+        <v>2</v>
+      </c>
+      <c r="N533" t="s">
+        <v>28</v>
+      </c>
+      <c r="O533" s="3"/>
+      <c r="P533" s="6">
+        <v>44384</v>
+      </c>
+      <c r="Q533" s="6">
+        <v>44229</v>
+      </c>
+      <c r="R533" s="6">
+        <v>44321</v>
+      </c>
+      <c r="S533" t="s">
+        <v>3257</v>
+      </c>
+      <c r="T533" s="5" t="s">
+        <v>3258</v>
+      </c>
+    </row>
+    <row r="534" spans="1:20" ht="15.75">
+      <c r="A534" t="s">
+        <v>3259</v>
+      </c>
+      <c r="B534" t="s">
+        <v>1466</v>
+      </c>
+      <c r="C534" t="s">
+        <v>3260</v>
+      </c>
+      <c r="D534" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E534" t="s">
+        <v>21</v>
+      </c>
+      <c r="F534" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G534" s="3">
+        <v>4</v>
+      </c>
+      <c r="H534" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I534" t="s">
+        <v>3261</v>
+      </c>
+      <c r="J534" t="s">
+        <v>8</v>
+      </c>
+      <c r="K534" t="s">
+        <v>37</v>
+      </c>
+      <c r="L534" s="3">
+        <v>1</v>
+      </c>
+      <c r="M534" s="3">
+        <v>4</v>
+      </c>
+      <c r="N534" t="s">
+        <v>28</v>
+      </c>
+      <c r="O534" s="3"/>
+      <c r="P534" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q534" s="3">
+        <v>2</v>
+      </c>
+      <c r="R534" s="3">
+        <v>4</v>
+      </c>
+      <c r="S534" t="s">
+        <v>794</v>
+      </c>
+      <c r="T534" s="5" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="535" spans="1:20" ht="15.75">
+      <c r="A535" t="s">
+        <v>3262</v>
+      </c>
+      <c r="B535" t="s">
+        <v>3263</v>
+      </c>
+      <c r="C535" t="s">
+        <v>3264</v>
+      </c>
+      <c r="D535" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E535" t="s">
+        <v>26</v>
+      </c>
+      <c r="F535" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G535" s="3">
+        <v>4</v>
+      </c>
+      <c r="H535" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I535" t="s">
+        <v>3265</v>
+      </c>
+      <c r="J535" t="s">
+        <v>8</v>
+      </c>
+      <c r="K535" t="s">
+        <v>47</v>
+      </c>
+      <c r="L535" s="3">
+        <v>2</v>
+      </c>
+      <c r="M535" s="3">
+        <v>3</v>
+      </c>
+      <c r="N535" t="s">
+        <v>23</v>
+      </c>
+      <c r="O535" s="3"/>
+      <c r="P535" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q535" s="3">
+        <v>1</v>
+      </c>
+      <c r="R535" s="3">
+        <v>5</v>
+      </c>
+      <c r="S535" t="s">
+        <v>790</v>
+      </c>
+      <c r="T535" s="5" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="536" spans="1:20" ht="15.75">
+      <c r="A536" t="s">
+        <v>3266</v>
+      </c>
+      <c r="B536" t="s">
+        <v>3267</v>
+      </c>
+      <c r="C536" t="s">
+        <v>3268</v>
+      </c>
+      <c r="D536" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E536" t="s">
+        <v>21</v>
+      </c>
+      <c r="F536" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G536" s="3">
+        <v>4</v>
+      </c>
+      <c r="H536" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I536" t="s">
+        <v>3269</v>
+      </c>
+      <c r="J536" t="s">
+        <v>287</v>
+      </c>
+      <c r="K536" t="s">
+        <v>905</v>
+      </c>
+      <c r="L536" s="3">
+        <v>5</v>
+      </c>
+      <c r="M536" s="3">
+        <v>2</v>
+      </c>
+      <c r="N536" t="s">
+        <v>292</v>
+      </c>
+      <c r="O536" s="3"/>
+      <c r="P536" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q536" s="3">
+        <v>5</v>
+      </c>
+      <c r="R536" s="3">
+        <v>4</v>
+      </c>
+      <c r="S536" t="s">
+        <v>3270</v>
+      </c>
+      <c r="T536" s="5" t="s">
+        <v>3271</v>
+      </c>
+    </row>
+    <row r="537" spans="1:20" ht="15.75">
+      <c r="A537" t="s">
+        <v>3272</v>
+      </c>
+      <c r="B537" t="s">
+        <v>1476</v>
+      </c>
+      <c r="C537" t="s">
+        <v>3273</v>
+      </c>
+      <c r="D537" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E537" t="s">
+        <v>21</v>
+      </c>
+      <c r="F537" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G537" s="3">
+        <v>4</v>
+      </c>
+      <c r="H537" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I537" t="s">
+        <v>3274</v>
+      </c>
+      <c r="J537" t="s">
+        <v>8</v>
+      </c>
+      <c r="K537" t="s">
+        <v>818</v>
+      </c>
+      <c r="L537" s="3">
+        <v>5</v>
+      </c>
+      <c r="M537" s="3">
+        <v>3</v>
+      </c>
+      <c r="N537" t="s">
+        <v>28</v>
+      </c>
+      <c r="O537" s="3"/>
+      <c r="P537" s="6">
+        <v>43892</v>
+      </c>
+      <c r="Q537" s="6">
+        <v>43925</v>
+      </c>
+      <c r="R537" s="6">
+        <v>43955</v>
+      </c>
+      <c r="S537" t="s">
+        <v>819</v>
+      </c>
+      <c r="T537" s="5" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="538" spans="1:20" ht="15.75">
+      <c r="A538" t="s">
+        <v>3275</v>
+      </c>
+      <c r="B538" t="s">
+        <v>3276</v>
+      </c>
+      <c r="C538" t="s">
+        <v>3277</v>
+      </c>
+      <c r="D538" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E538" t="s">
+        <v>21</v>
+      </c>
+      <c r="F538" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G538" s="3">
+        <v>4</v>
+      </c>
+      <c r="H538" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I538" t="s">
+        <v>3278</v>
+      </c>
+      <c r="J538" t="s">
+        <v>8</v>
+      </c>
+      <c r="K538" t="s">
+        <v>811</v>
+      </c>
+      <c r="L538" s="3">
+        <v>2</v>
+      </c>
+      <c r="M538" s="3">
+        <v>2</v>
+      </c>
+      <c r="N538" t="s">
+        <v>11</v>
+      </c>
+      <c r="O538" s="3"/>
+      <c r="P538" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q538" s="3">
+        <v>1</v>
+      </c>
+      <c r="R538" s="3">
+        <v>4</v>
+      </c>
+      <c r="S538" t="s">
+        <v>812</v>
+      </c>
+      <c r="T538" s="5" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="539" spans="1:20" ht="15.75">
+      <c r="A539" t="s">
+        <v>3279</v>
+      </c>
+      <c r="B539" t="s">
+        <v>1478</v>
+      </c>
+      <c r="C539" t="s">
+        <v>3280</v>
+      </c>
+      <c r="D539" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E539" t="s">
+        <v>21</v>
+      </c>
+      <c r="F539" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G539" s="3">
+        <v>4</v>
+      </c>
+      <c r="H539" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I539" t="s">
+        <v>3281</v>
+      </c>
+      <c r="J539" t="s">
+        <v>8</v>
+      </c>
+      <c r="K539" t="s">
+        <v>824</v>
+      </c>
+      <c r="L539" s="3">
+        <v>2</v>
+      </c>
+      <c r="M539" s="3">
+        <v>4</v>
+      </c>
+      <c r="N539" t="s">
+        <v>11</v>
+      </c>
+      <c r="O539" s="3"/>
+      <c r="P539" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q539" s="3">
+        <v>2</v>
+      </c>
+      <c r="R539" s="3">
+        <v>4</v>
+      </c>
+      <c r="S539" t="s">
+        <v>825</v>
+      </c>
+      <c r="T539" s="5" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="540" spans="1:20" ht="15.75">
+      <c r="A540" t="s">
+        <v>3282</v>
+      </c>
+      <c r="B540" t="s">
+        <v>1482</v>
+      </c>
+      <c r="C540" t="s">
+        <v>3283</v>
+      </c>
+      <c r="D540" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E540" t="s">
+        <v>26</v>
+      </c>
+      <c r="F540" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G540" s="3">
+        <v>4</v>
+      </c>
+      <c r="H540" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I540" t="s">
+        <v>3284</v>
+      </c>
+      <c r="J540" t="s">
+        <v>8</v>
+      </c>
+      <c r="K540" t="s">
+        <v>142</v>
+      </c>
+      <c r="L540" s="3">
+        <v>2</v>
+      </c>
+      <c r="M540" s="3">
+        <v>3</v>
+      </c>
+      <c r="N540" t="s">
+        <v>28</v>
+      </c>
+      <c r="O540" s="3"/>
+      <c r="P540" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q540" s="3">
+        <v>1</v>
+      </c>
+      <c r="R540" s="3">
+        <v>5</v>
+      </c>
+      <c r="S540" t="s">
+        <v>834</v>
+      </c>
+      <c r="T540" s="5" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="541" spans="1:20" ht="15.75">
+      <c r="A541" t="s">
+        <v>3285</v>
+      </c>
+      <c r="B541" t="s">
+        <v>1484</v>
+      </c>
+      <c r="C541" t="s">
+        <v>3286</v>
+      </c>
+      <c r="D541" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E541" t="s">
+        <v>14</v>
+      </c>
+      <c r="F541" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G541" s="3">
+        <v>4</v>
+      </c>
+      <c r="H541" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I541" t="s">
+        <v>3287</v>
+      </c>
+      <c r="J541" t="s">
+        <v>8</v>
+      </c>
+      <c r="K541" t="s">
+        <v>18</v>
+      </c>
+      <c r="L541" s="3">
+        <v>0</v>
+      </c>
+      <c r="M541" s="3">
+        <v>6</v>
+      </c>
+      <c r="N541" t="s">
+        <v>28</v>
+      </c>
+      <c r="O541" s="3"/>
+      <c r="P541" s="3"/>
+      <c r="Q541" s="3"/>
+      <c r="R541" s="3"/>
+      <c r="S541" t="s">
+        <v>839</v>
+      </c>
+      <c r="T541" s="5" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="542" spans="1:20" ht="15.75">
+      <c r="A542" t="s">
+        <v>3288</v>
+      </c>
+      <c r="B542" t="s">
+        <v>3289</v>
+      </c>
+      <c r="C542" t="s">
+        <v>3290</v>
+      </c>
+      <c r="D542" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E542" t="s">
+        <v>79</v>
+      </c>
+      <c r="F542" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G542" s="3">
+        <v>4</v>
+      </c>
+      <c r="H542" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I542" t="s">
+        <v>3291</v>
+      </c>
+      <c r="J542" t="s">
+        <v>287</v>
+      </c>
+      <c r="K542" t="s">
+        <v>327</v>
+      </c>
+      <c r="L542" s="3">
+        <v>4</v>
+      </c>
+      <c r="M542" s="3">
+        <v>2</v>
+      </c>
+      <c r="N542" t="s">
+        <v>304</v>
+      </c>
+      <c r="O542" s="3"/>
+      <c r="P542" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q542" s="3">
+        <v>1</v>
+      </c>
+      <c r="R542" s="3">
+        <v>3</v>
+      </c>
+      <c r="S542" t="s">
+        <v>968</v>
+      </c>
+      <c r="T542" s="5" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="543" spans="1:20" ht="15.75">
+      <c r="A543" t="s">
+        <v>3292</v>
+      </c>
+      <c r="B543" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C543" t="s">
+        <v>3293</v>
+      </c>
+      <c r="D543" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E543" t="s">
+        <v>21</v>
+      </c>
+      <c r="F543" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G543" s="3">
+        <v>4</v>
+      </c>
+      <c r="H543" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I543" t="s">
+        <v>3294</v>
+      </c>
+      <c r="J543" t="s">
+        <v>149</v>
+      </c>
+      <c r="K543" t="s">
+        <v>841</v>
+      </c>
+      <c r="L543" s="3">
+        <v>3</v>
+      </c>
+      <c r="M543" s="3">
+        <v>1</v>
+      </c>
+      <c r="N543" t="s">
+        <v>150</v>
+      </c>
+      <c r="O543" s="3"/>
+      <c r="P543" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q543" s="3">
+        <v>3</v>
+      </c>
+      <c r="R543" s="3">
+        <v>4</v>
+      </c>
+      <c r="S543" t="s">
+        <v>842</v>
+      </c>
+      <c r="T543" s="5" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="544" spans="1:20" ht="15.75">
+      <c r="A544" t="s">
+        <v>3295</v>
+      </c>
+      <c r="B544" t="s">
+        <v>3296</v>
+      </c>
+      <c r="C544" t="s">
+        <v>3297</v>
+      </c>
+      <c r="D544" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E544" t="s">
+        <v>14</v>
+      </c>
+      <c r="F544" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G544" s="3">
+        <v>4</v>
+      </c>
+      <c r="H544" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I544" t="s">
+        <v>3298</v>
+      </c>
+      <c r="J544" t="s">
+        <v>426</v>
+      </c>
+      <c r="K544" t="s">
+        <v>15</v>
+      </c>
+      <c r="L544" s="3">
+        <v>0</v>
+      </c>
+      <c r="M544" s="3">
+        <v>5</v>
+      </c>
+      <c r="N544" t="s">
+        <v>428</v>
+      </c>
+      <c r="O544" s="3"/>
+      <c r="P544" s="3"/>
+      <c r="Q544" s="3"/>
+      <c r="R544" s="3"/>
+      <c r="S544" t="s">
+        <v>983</v>
+      </c>
+      <c r="T544" s="5" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="545" spans="1:20" ht="15.75">
+      <c r="A545" t="s">
+        <v>3299</v>
+      </c>
+      <c r="B545" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C545" t="s">
+        <v>3300</v>
+      </c>
+      <c r="D545" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E545" t="s">
+        <v>176</v>
+      </c>
+      <c r="F545" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G545" s="3">
+        <v>4</v>
+      </c>
+      <c r="H545" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I545" t="s">
+        <v>3301</v>
+      </c>
+      <c r="J545" t="s">
+        <v>149</v>
+      </c>
+      <c r="K545" t="s">
+        <v>3302</v>
+      </c>
+      <c r="L545" s="3">
+        <v>5</v>
+      </c>
+      <c r="M545" s="3">
+        <v>4</v>
+      </c>
+      <c r="N545" t="s">
+        <v>158</v>
+      </c>
+      <c r="O545" s="3"/>
+      <c r="P545" s="6">
+        <v>43931</v>
+      </c>
+      <c r="Q545" s="6">
+        <v>43892</v>
+      </c>
+      <c r="R545" s="6">
+        <v>44109</v>
+      </c>
+      <c r="S545" t="s">
+        <v>859</v>
+      </c>
+      <c r="T545" s="5" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="546" spans="1:20" ht="15.75">
+      <c r="A546" t="s">
+        <v>3303</v>
+      </c>
+      <c r="B546" t="s">
+        <v>3304</v>
+      </c>
+      <c r="C546" t="s">
+        <v>3305</v>
+      </c>
+      <c r="D546" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E546" t="s">
+        <v>21</v>
+      </c>
+      <c r="F546" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G546" s="3">
+        <v>4</v>
+      </c>
+      <c r="H546" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I546" t="s">
+        <v>3306</v>
+      </c>
+      <c r="J546" t="s">
+        <v>426</v>
+      </c>
+      <c r="K546" t="s">
+        <v>1001</v>
+      </c>
+      <c r="L546" s="3">
+        <v>1</v>
+      </c>
+      <c r="M546" s="3">
+        <v>3</v>
+      </c>
+      <c r="N546" t="s">
+        <v>435</v>
+      </c>
+      <c r="O546" s="3"/>
+      <c r="P546" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q546" s="3">
+        <v>1</v>
+      </c>
+      <c r="R546" s="3">
+        <v>3</v>
+      </c>
+      <c r="S546" t="s">
+        <v>1002</v>
+      </c>
+      <c r="T546" s="5" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="547" spans="1:20" ht="15.75">
+      <c r="A547" t="s">
+        <v>3307</v>
+      </c>
+      <c r="B547" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C547" t="s">
+        <v>3308</v>
+      </c>
+      <c r="D547" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E547" t="s">
+        <v>14</v>
+      </c>
+      <c r="F547" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G547" s="3">
+        <v>4</v>
+      </c>
+      <c r="H547" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I547" t="s">
+        <v>3309</v>
+      </c>
+      <c r="J547" t="s">
+        <v>149</v>
+      </c>
+      <c r="K547" t="s">
+        <v>18</v>
+      </c>
+      <c r="L547" s="3">
+        <v>1</v>
+      </c>
+      <c r="M547" s="3">
+        <v>4</v>
+      </c>
+      <c r="N547" t="s">
+        <v>150</v>
+      </c>
+      <c r="O547" s="3"/>
+      <c r="P547" s="3"/>
+      <c r="Q547" s="3"/>
+      <c r="R547" s="3"/>
+      <c r="S547" t="s">
+        <v>881</v>
+      </c>
+      <c r="T547" s="5" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="548" spans="1:20" ht="15.75">
+      <c r="A548" t="s">
+        <v>3310</v>
+      </c>
+      <c r="B548" t="s">
+        <v>3311</v>
+      </c>
+      <c r="C548" t="s">
+        <v>3312</v>
+      </c>
+      <c r="D548" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E548" t="s">
+        <v>21</v>
+      </c>
+      <c r="F548" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G548" s="3">
+        <v>4</v>
+      </c>
+      <c r="H548" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I548" t="s">
+        <v>3313</v>
+      </c>
+      <c r="J548" t="s">
+        <v>557</v>
+      </c>
+      <c r="K548" t="s">
+        <v>1061</v>
+      </c>
+      <c r="L548" s="3">
+        <v>2</v>
+      </c>
+      <c r="M548" s="3">
+        <v>4</v>
+      </c>
+      <c r="N548" t="s">
+        <v>558</v>
+      </c>
+      <c r="O548" s="3"/>
+      <c r="P548" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q548" s="3">
+        <v>1</v>
+      </c>
+      <c r="R548" s="3">
+        <v>3</v>
+      </c>
+      <c r="S548" t="s">
+        <v>1076</v>
+      </c>
+      <c r="T548" s="5" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="549" spans="1:20" ht="15.75">
+      <c r="A549" t="s">
+        <v>3314</v>
+      </c>
+      <c r="B549" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C549" t="s">
+        <v>3315</v>
+      </c>
+      <c r="D549" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E549" t="s">
+        <v>21</v>
+      </c>
+      <c r="F549" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G549" s="3">
+        <v>4</v>
+      </c>
+      <c r="H549" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I549" t="s">
+        <v>3316</v>
+      </c>
+      <c r="J549" t="s">
+        <v>149</v>
+      </c>
+      <c r="K549" t="s">
+        <v>180</v>
+      </c>
+      <c r="L549" s="3">
+        <v>4</v>
+      </c>
+      <c r="M549" s="3">
+        <v>1</v>
+      </c>
+      <c r="N549" t="s">
+        <v>158</v>
+      </c>
+      <c r="O549" s="3"/>
+      <c r="P549" s="3">
+        <v>5</v>
+      </c>
+      <c r="Q549" s="3">
+        <v>3</v>
+      </c>
+      <c r="R549" s="3">
+        <v>4</v>
+      </c>
+      <c r="S549" t="s">
+        <v>885</v>
+      </c>
+      <c r="T549" s="5" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="550" spans="1:20" ht="15.75">
+      <c r="A550" t="s">
+        <v>3317</v>
+      </c>
+      <c r="B550" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C550" t="s">
+        <v>3318</v>
+      </c>
+      <c r="D550" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E550" t="s">
+        <v>21</v>
+      </c>
+      <c r="F550" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G550" s="3">
+        <v>4</v>
+      </c>
+      <c r="H550" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I550" t="s">
+        <v>3319</v>
+      </c>
+      <c r="J550" t="s">
+        <v>149</v>
+      </c>
+      <c r="K550" t="s">
+        <v>222</v>
+      </c>
+      <c r="L550" s="3">
+        <v>4</v>
+      </c>
+      <c r="M550" s="3">
+        <v>4</v>
+      </c>
+      <c r="N550" t="s">
+        <v>158</v>
+      </c>
+      <c r="O550" s="3"/>
+      <c r="P550" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q550" s="3">
+        <v>4</v>
+      </c>
+      <c r="R550" s="3">
+        <v>4</v>
+      </c>
+      <c r="S550" t="s">
+        <v>891</v>
+      </c>
+      <c r="T550" s="5" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="551" spans="1:20" ht="15.75">
+      <c r="A551" t="s">
+        <v>3320</v>
+      </c>
+      <c r="B551" t="s">
+        <v>1511</v>
+      </c>
+      <c r="C551" t="s">
+        <v>3321</v>
+      </c>
+      <c r="D551" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E551" t="s">
+        <v>153</v>
+      </c>
+      <c r="F551" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G551" s="3">
+        <v>4</v>
+      </c>
+      <c r="H551" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I551" t="s">
+        <v>3322</v>
+      </c>
+      <c r="J551" t="s">
+        <v>149</v>
+      </c>
+      <c r="K551" t="s">
+        <v>154</v>
+      </c>
+      <c r="L551" s="3">
+        <v>2</v>
+      </c>
+      <c r="M551" s="3">
+        <v>6</v>
+      </c>
+      <c r="N551" t="s">
+        <v>158</v>
+      </c>
+      <c r="O551" s="3"/>
+      <c r="P551" s="3"/>
+      <c r="Q551" s="3"/>
+      <c r="R551" s="3"/>
+      <c r="S551" t="s">
+        <v>899</v>
+      </c>
+      <c r="T551" s="5" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="552" spans="1:20" ht="15.75">
+      <c r="A552" t="s">
+        <v>3323</v>
+      </c>
+      <c r="B552" t="s">
+        <v>3324</v>
+      </c>
+      <c r="C552" t="s">
+        <v>3325</v>
+      </c>
+      <c r="D552" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E552" t="s">
+        <v>26</v>
+      </c>
+      <c r="F552" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G552" s="3">
+        <v>4</v>
+      </c>
+      <c r="H552" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I552" t="s">
+        <v>3326</v>
+      </c>
+      <c r="J552" t="s">
+        <v>557</v>
+      </c>
+      <c r="K552" t="s">
+        <v>1086</v>
+      </c>
+      <c r="L552" s="3">
+        <v>4</v>
+      </c>
+      <c r="M552" s="3">
+        <v>2</v>
+      </c>
+      <c r="N552" t="s">
+        <v>558</v>
+      </c>
+      <c r="O552" s="3"/>
+      <c r="P552" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q552" s="3">
+        <v>2</v>
+      </c>
+      <c r="R552" s="3">
+        <v>5</v>
+      </c>
+      <c r="S552" t="s">
+        <v>1087</v>
+      </c>
+      <c r="T552" s="5" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="553" spans="1:20" ht="15.75">
+      <c r="A553" t="s">
+        <v>3327</v>
+      </c>
+      <c r="B553" t="s">
+        <v>1514</v>
+      </c>
+      <c r="C553" t="s">
+        <v>3328</v>
+      </c>
+      <c r="D553" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E553" t="s">
+        <v>21</v>
+      </c>
+      <c r="F553" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G553" s="3">
+        <v>4</v>
+      </c>
+      <c r="H553" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I553" t="s">
+        <v>3329</v>
+      </c>
+      <c r="J553" t="s">
+        <v>287</v>
+      </c>
+      <c r="K553" t="s">
+        <v>905</v>
+      </c>
+      <c r="L553" s="3">
+        <v>3</v>
+      </c>
+      <c r="M553" s="3">
+        <v>5</v>
+      </c>
+      <c r="N553" t="s">
+        <v>292</v>
+      </c>
+      <c r="O553" s="3"/>
+      <c r="P553" s="3">
+        <v>3</v>
+      </c>
+      <c r="Q553" s="3">
+        <v>2</v>
+      </c>
+      <c r="R553" s="3">
+        <v>4</v>
+      </c>
+      <c r="S553" t="s">
+        <v>906</v>
+      </c>
+      <c r="T553" s="5" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="554" spans="1:20" ht="15.75">
+      <c r="A554" t="s">
+        <v>3330</v>
+      </c>
+      <c r="B554" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C554" t="s">
+        <v>3331</v>
+      </c>
+      <c r="D554" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E554" t="s">
+        <v>26</v>
+      </c>
+      <c r="F554" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G554" s="3">
+        <v>4</v>
+      </c>
+      <c r="H554" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I554" t="s">
+        <v>3332</v>
+      </c>
+      <c r="J554" t="s">
+        <v>287</v>
+      </c>
+      <c r="K554" t="s">
+        <v>915</v>
+      </c>
+      <c r="L554" s="3">
+        <v>3</v>
+      </c>
+      <c r="M554" s="3">
+        <v>2</v>
+      </c>
+      <c r="N554" t="s">
+        <v>292</v>
+      </c>
+      <c r="O554" s="3"/>
+      <c r="P554" s="6">
+        <v>43865</v>
+      </c>
+      <c r="Q554" s="6">
+        <v>43831</v>
+      </c>
+      <c r="R554" s="6">
+        <v>43956</v>
+      </c>
+      <c r="S554" t="s">
+        <v>916</v>
+      </c>
+      <c r="T554" s="5" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="555" spans="1:20" ht="15.75">
+      <c r="A555" t="s">
+        <v>3333</v>
+      </c>
+      <c r="B555" t="s">
+        <v>1529</v>
+      </c>
+      <c r="C555" t="s">
+        <v>3334</v>
+      </c>
+      <c r="D555" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E555" t="s">
+        <v>21</v>
+      </c>
+      <c r="F555" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G555" s="3">
+        <v>4</v>
+      </c>
+      <c r="H555" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I555" t="s">
+        <v>3335</v>
+      </c>
+      <c r="J555" t="s">
+        <v>287</v>
+      </c>
+      <c r="K555" t="s">
+        <v>407</v>
+      </c>
+      <c r="L555" s="3">
+        <v>3</v>
+      </c>
+      <c r="M555" s="3">
+        <v>2</v>
+      </c>
+      <c r="N555" t="s">
+        <v>292</v>
+      </c>
+      <c r="O555" s="3"/>
+      <c r="P555" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q555" s="3">
+        <v>4</v>
+      </c>
+      <c r="R555" s="3">
+        <v>5</v>
+      </c>
+      <c r="S555" t="s">
+        <v>943</v>
+      </c>
+      <c r="T555" s="5" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="556" spans="1:20" ht="15.75">
+      <c r="A556" t="s">
+        <v>3336</v>
+      </c>
+      <c r="B556" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C556" t="s">
+        <v>3337</v>
+      </c>
+      <c r="D556" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E556" t="s">
+        <v>9</v>
+      </c>
+      <c r="F556" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G556" s="3">
+        <v>4</v>
+      </c>
+      <c r="H556" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I556" t="s">
+        <v>3338</v>
+      </c>
+      <c r="J556" t="s">
+        <v>287</v>
+      </c>
+      <c r="K556" t="s">
+        <v>796</v>
+      </c>
+      <c r="L556" s="3">
+        <v>2</v>
+      </c>
+      <c r="M556" s="3">
+        <v>7</v>
+      </c>
+      <c r="N556" t="s">
+        <v>292</v>
+      </c>
+      <c r="O556" s="3"/>
+      <c r="P556" s="3"/>
+      <c r="Q556" s="3"/>
+      <c r="R556" s="3"/>
+      <c r="S556" t="s">
+        <v>945</v>
+      </c>
+      <c r="T556" s="5" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="557" spans="1:20" ht="15.75">
+      <c r="A557" t="s">
+        <v>3339</v>
+      </c>
+      <c r="B557" t="s">
+        <v>1532</v>
+      </c>
+      <c r="C557" t="s">
+        <v>3340</v>
+      </c>
+      <c r="D557" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E557" t="s">
+        <v>14</v>
+      </c>
+      <c r="F557" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G557" s="3">
+        <v>4</v>
+      </c>
+      <c r="H557" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I557" t="s">
+        <v>3341</v>
+      </c>
+      <c r="J557" t="s">
+        <v>287</v>
+      </c>
+      <c r="K557" t="s">
+        <v>18</v>
+      </c>
+      <c r="L557" s="3">
+        <v>1</v>
+      </c>
+      <c r="M557" s="3">
+        <v>3</v>
+      </c>
+      <c r="N557" t="s">
+        <v>288</v>
+      </c>
+      <c r="O557" s="3"/>
+      <c r="P557" s="3"/>
+      <c r="Q557" s="3"/>
+      <c r="R557" s="3"/>
+      <c r="S557" t="s">
+        <v>949</v>
+      </c>
+      <c r="T557" s="5" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="558" spans="1:20" ht="15.75">
+      <c r="A558" t="s">
+        <v>3342</v>
+      </c>
+      <c r="B558" t="s">
+        <v>1551</v>
+      </c>
+      <c r="C558" t="s">
+        <v>3343</v>
+      </c>
+      <c r="D558" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E558" t="s">
+        <v>21</v>
+      </c>
+      <c r="F558" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G558" s="3">
+        <v>4</v>
+      </c>
+      <c r="H558" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I558" t="s">
+        <v>3344</v>
+      </c>
+      <c r="J558" t="s">
+        <v>426</v>
+      </c>
+      <c r="K558" t="s">
+        <v>989</v>
+      </c>
+      <c r="L558" s="3">
+        <v>2</v>
+      </c>
+      <c r="M558" s="3">
+        <v>7</v>
+      </c>
+      <c r="N558" t="s">
+        <v>448</v>
+      </c>
+      <c r="O558" s="3"/>
+      <c r="P558" s="3">
+        <v>4</v>
+      </c>
+      <c r="Q558" s="3">
+        <v>5</v>
+      </c>
+      <c r="R558" s="3">
+        <v>4</v>
+      </c>
+      <c r="S558" t="s">
+        <v>990</v>
+      </c>
+      <c r="T558" s="5" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="559" spans="1:20" ht="15.75">
+      <c r="A559" t="s">
+        <v>3345</v>
+      </c>
+      <c r="B559" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C559" t="s">
+        <v>3346</v>
+      </c>
+      <c r="D559" t="s">
+        <v>3101</v>
+      </c>
+      <c r="E559" t="s">
+        <v>14</v>
+      </c>
+      <c r="F559" s="3" t="s">
+        <v>2113</v>
+      </c>
+      <c r="G559" s="3">
+        <v>4</v>
+      </c>
+      <c r="H559" t="s">
+        <v>3097</v>
+      </c>
+      <c r="I559" t="s">
+        <v>3347</v>
+      </c>
+      <c r="J559" t="s">
+        <v>557</v>
+      </c>
+      <c r="K559" t="s">
+        <v>18</v>
+      </c>
+      <c r="L559" s="3">
+        <v>0</v>
+      </c>
+      <c r="M559" s="3">
+        <v>6</v>
+      </c>
+      <c r="N559" t="s">
+        <v>573</v>
+      </c>
+      <c r="O559" s="3"/>
+      <c r="P559" s="3"/>
+      <c r="Q559" s="3"/>
+      <c r="R559" s="3"/>
+      <c r="S559" t="s">
+        <v>1080</v>
+      </c>
+      <c r="T559" s="5" t="s">
+        <v>1081</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T492" xr:uid="{48FE8A57-0D3F-49E0-BA7C-D0804C020F31}"/>
+  <hyperlinks>
+    <hyperlink ref="C493" r:id="rId1" display="https://warstcg.org//img/1/WARS-EN01001.jpg" xr:uid="{B6B8140D-9AF2-4F5E-B513-6FCDD67CA049}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>